<commit_message>
Fix Excel card master and filters
</commit_message>
<xml_diff>
--- a/card_master.xlsx
+++ b/card_master.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\平石　美帆\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\平石　美帆\aikatsu-encore-manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{CF61352F-56D6-4381-AE32-CEC0E32BEDDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{971C5BD4-EA63-432E-AA50-F41212D003B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="358">
   <si>
     <t>カード番号</t>
   </si>
@@ -1259,6 +1259,13 @@
   </si>
   <si>
     <t>イエローブロッサムコーデ</t>
+    <phoneticPr fontId="5"/>
+  </si>
+  <si>
+    <t>第一弾</t>
+    <rPh sb="0" eb="3">
+      <t>ダイイチダン</t>
+    </rPh>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1387,10 +1394,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1401,6 +1404,10 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1775,15 +1782,15 @@
         <v>14</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E2" t="s">
         <v>233</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H2" s="5" t="s">
@@ -1815,15 +1822,15 @@
         <v>14</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E3" t="s">
         <v>233</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H3" s="5" t="s">
@@ -1855,15 +1862,15 @@
         <v>14</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E4" t="s">
         <v>233</v>
       </c>
-      <c r="F4" s="11" t="s">
+      <c r="F4" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H4" s="5" t="s">
@@ -1891,15 +1898,15 @@
         <v>14</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E5" t="s">
         <v>233</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H5" s="5" t="s">
@@ -1920,22 +1927,22 @@
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>234</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E6" t="s">
         <v>238</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H6" s="5" t="s">
@@ -1956,22 +1963,22 @@
       <c r="A7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="10" t="s">
         <v>235</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E7" t="s">
         <v>238</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H7" s="5" t="s">
@@ -1992,22 +1999,22 @@
       <c r="A8" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="10" t="s">
         <v>236</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E8" t="s">
         <v>238</v>
       </c>
-      <c r="F8" s="11" t="s">
+      <c r="F8" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H8" s="5" t="s">
@@ -2035,15 +2042,15 @@
         <v>27</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E9" t="s">
         <v>238</v>
       </c>
-      <c r="F9" s="11" t="s">
+      <c r="F9" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H9" s="5" t="s">
@@ -2071,15 +2078,15 @@
         <v>27</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E10" t="s">
         <v>240</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H10" s="5" t="s">
@@ -2107,15 +2114,15 @@
         <v>27</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E11" t="s">
         <v>246</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H11" s="5" t="s">
@@ -2143,15 +2150,15 @@
         <v>27</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E12" t="s">
         <v>246</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H12" s="5" t="s">
@@ -2179,15 +2186,15 @@
         <v>27</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E13" t="s">
         <v>246</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H13" s="5" t="s">
@@ -2215,15 +2222,15 @@
         <v>27</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E14" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H14" s="5" t="s">
@@ -2251,15 +2258,15 @@
         <v>27</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E15" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E15" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G15" s="11" t="s">
+      <c r="G15" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H15" s="5" t="s">
@@ -2287,15 +2294,15 @@
         <v>27</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E16" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="F16" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H16" s="5" t="s">
@@ -2323,15 +2330,15 @@
         <v>27</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E17" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>251</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G17" s="11" t="s">
+      <c r="G17" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H17" s="5" t="s">
@@ -2359,15 +2366,15 @@
         <v>27</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E18" t="s">
         <v>257</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G18" s="11" t="s">
+      <c r="G18" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H18" s="5" t="s">
@@ -2388,22 +2395,22 @@
       <c r="A19" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="10" t="s">
         <v>254</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E19" t="s">
         <v>257</v>
       </c>
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G19" s="11" t="s">
+      <c r="G19" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H19" s="5" t="s">
@@ -2431,15 +2438,15 @@
         <v>27</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E20" t="s">
         <v>257</v>
       </c>
-      <c r="F20" s="11" t="s">
+      <c r="F20" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G20" s="11" t="s">
+      <c r="G20" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H20" s="5" t="s">
@@ -2467,15 +2474,15 @@
         <v>27</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E21" t="s">
         <v>257</v>
       </c>
-      <c r="F21" s="11" t="s">
+      <c r="F21" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G21" s="11" t="s">
+      <c r="G21" s="9" t="s">
         <v>241</v>
       </c>
       <c r="H21" s="5" t="s">
@@ -2503,15 +2510,15 @@
         <v>60</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E22" t="s">
         <v>260</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H22" s="5" t="s">
@@ -2539,15 +2546,15 @@
         <v>60</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E23" t="s">
         <v>260</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G23" s="11" t="s">
+      <c r="G23" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H23" s="5" t="s">
@@ -2575,15 +2582,15 @@
         <v>60</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E24" t="s">
         <v>260</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H24" s="5" t="s">
@@ -2611,18 +2618,18 @@
         <v>60</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E25" t="s">
         <v>265</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="G25" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="H25" s="13" t="s">
+      <c r="H25" s="11" t="s">
         <v>271</v>
       </c>
       <c r="I25" s="4" t="s">
@@ -2647,15 +2654,15 @@
         <v>60</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E26" t="s">
         <v>265</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G26" s="11" t="s">
+      <c r="G26" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H26" s="5" t="s">
@@ -2683,15 +2690,15 @@
         <v>60</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E27" t="s">
         <v>265</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F27" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G27" s="11" t="s">
+      <c r="G27" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H27" s="5" t="s">
@@ -2719,18 +2726,18 @@
         <v>60</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E28" t="s">
         <v>270</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G28" s="11" t="s">
+      <c r="G28" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="H28" s="13" t="s">
+      <c r="H28" s="11" t="s">
         <v>271</v>
       </c>
       <c r="I28" s="4" t="s">
@@ -2755,15 +2762,15 @@
         <v>60</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E29" t="s">
         <v>270</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="F29" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="G29" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H29" s="5" t="s">
@@ -2791,15 +2798,15 @@
         <v>60</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E30" t="s">
         <v>270</v>
       </c>
-      <c r="F30" s="11" t="s">
+      <c r="F30" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G30" s="11" t="s">
+      <c r="G30" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H30" s="5" t="s">
@@ -2827,15 +2834,15 @@
         <v>79</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E31" t="s">
         <v>273</v>
       </c>
-      <c r="F31" s="11" t="s">
+      <c r="F31" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G31" s="11" t="s">
+      <c r="G31" s="9" t="s">
         <v>247</v>
       </c>
       <c r="H31" s="5" t="s">
@@ -2863,15 +2870,15 @@
         <v>79</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E32" t="s">
         <v>275</v>
       </c>
-      <c r="F32" s="11" t="s">
+      <c r="F32" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G32" s="11" t="s">
+      <c r="G32" s="9" t="s">
         <v>276</v>
       </c>
       <c r="H32" s="5" t="s">
@@ -2899,15 +2906,15 @@
         <v>79</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E33" t="s">
         <v>278</v>
       </c>
-      <c r="F33" s="11" t="s">
+      <c r="F33" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="G33" s="11" t="s">
+      <c r="G33" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H33" s="5" t="s">
@@ -2935,15 +2942,15 @@
         <v>14</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E34" t="s">
         <v>280</v>
       </c>
-      <c r="F34" s="11" t="s">
+      <c r="F34" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G34" s="11" t="s">
+      <c r="G34" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H34" s="5" t="s">
@@ -2971,15 +2978,15 @@
         <v>14</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E35" t="s">
         <v>280</v>
       </c>
-      <c r="F35" s="11" t="s">
+      <c r="F35" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G35" s="11" t="s">
+      <c r="G35" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H35" s="5" t="s">
@@ -3007,15 +3014,15 @@
         <v>14</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E36" t="s">
         <v>280</v>
       </c>
-      <c r="F36" s="11" t="s">
+      <c r="F36" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G36" s="11" t="s">
+      <c r="G36" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H36" s="5" t="s">
@@ -3043,15 +3050,15 @@
         <v>14</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E37" t="s">
         <v>280</v>
       </c>
-      <c r="F37" s="11" t="s">
+      <c r="F37" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G37" s="11" t="s">
+      <c r="G37" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H37" s="5" t="s">
@@ -3079,15 +3086,15 @@
         <v>27</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E38" t="s">
         <v>287</v>
       </c>
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G38" s="11" t="s">
+      <c r="G38" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H38" s="5" t="s">
@@ -3115,15 +3122,15 @@
         <v>27</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E39" t="s">
         <v>289</v>
       </c>
-      <c r="F39" s="11" t="s">
+      <c r="F39" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G39" s="11" t="s">
+      <c r="G39" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H39" s="5" t="s">
@@ -3151,15 +3158,15 @@
         <v>27</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E40" t="s">
         <v>289</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="F40" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G40" s="11" t="s">
+      <c r="G40" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H40" s="5" t="s">
@@ -3187,15 +3194,15 @@
         <v>27</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E41" t="s">
         <v>289</v>
       </c>
-      <c r="F41" s="11" t="s">
+      <c r="F41" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G41" s="11" t="s">
+      <c r="G41" s="9" t="s">
         <v>281</v>
       </c>
       <c r="H41" s="5" t="s">
@@ -3223,15 +3230,15 @@
         <v>60</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E42" t="s">
         <v>295</v>
       </c>
-      <c r="F42" s="11" t="s">
+      <c r="F42" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G42" s="11" t="s">
+      <c r="G42" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H42" s="5" t="s">
@@ -3259,15 +3266,15 @@
         <v>60</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E43" t="s">
         <v>295</v>
       </c>
-      <c r="F43" s="11" t="s">
+      <c r="F43" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G43" s="11" t="s">
+      <c r="G43" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H43" s="5" t="s">
@@ -3295,15 +3302,15 @@
         <v>60</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E44" t="s">
         <v>295</v>
       </c>
-      <c r="F44" s="11" t="s">
+      <c r="F44" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G44" s="11" t="s">
+      <c r="G44" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H44" s="5" t="s">
@@ -3331,15 +3338,15 @@
         <v>60</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E45" t="s">
         <v>298</v>
       </c>
-      <c r="F45" s="11" t="s">
+      <c r="F45" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G45" s="11" t="s">
+      <c r="G45" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H45" s="5" t="s">
@@ -3367,15 +3374,15 @@
         <v>60</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E46" t="s">
         <v>298</v>
       </c>
-      <c r="F46" s="11" t="s">
+      <c r="F46" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G46" s="11" t="s">
+      <c r="G46" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H46" s="5" t="s">
@@ -3403,15 +3410,15 @@
         <v>60</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E47" t="s">
         <v>298</v>
       </c>
-      <c r="F47" s="11" t="s">
+      <c r="F47" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G47" s="11" t="s">
+      <c r="G47" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H47" s="5" t="s">
@@ -3439,15 +3446,15 @@
         <v>60</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E48" t="s">
         <v>303</v>
       </c>
-      <c r="F48" s="11" t="s">
+      <c r="F48" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G48" s="11" t="s">
+      <c r="G48" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H48" s="5" t="s">
@@ -3475,15 +3482,15 @@
         <v>60</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E49" t="s">
         <v>303</v>
       </c>
-      <c r="F49" s="11" t="s">
+      <c r="F49" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G49" s="11" t="s">
+      <c r="G49" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H49" s="5" t="s">
@@ -3511,15 +3518,15 @@
         <v>60</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E50" t="s">
         <v>303</v>
       </c>
-      <c r="F50" s="11" t="s">
+      <c r="F50" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G50" s="11" t="s">
+      <c r="G50" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H50" s="5" t="s">
@@ -3547,15 +3554,15 @@
         <v>79</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E51" t="s">
         <v>305</v>
       </c>
-      <c r="F51" s="11" t="s">
+      <c r="F51" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="G51" s="11" t="s">
+      <c r="G51" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H51" s="5" t="s">
@@ -3583,15 +3590,15 @@
         <v>14</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E52" t="s">
         <v>307</v>
       </c>
-      <c r="F52" s="11" t="s">
+      <c r="F52" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G52" s="11" t="s">
+      <c r="G52" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H52" s="5" t="s">
@@ -3619,15 +3626,15 @@
         <v>14</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E53" t="s">
         <v>307</v>
       </c>
-      <c r="F53" s="11" t="s">
+      <c r="F53" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G53" s="11" t="s">
+      <c r="G53" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H53" s="5" t="s">
@@ -3655,15 +3662,15 @@
         <v>27</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E54" t="s">
         <v>311</v>
       </c>
-      <c r="F54" s="11" t="s">
+      <c r="F54" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G54" s="11" t="s">
+      <c r="G54" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H54" s="5" t="s">
@@ -3691,15 +3698,15 @@
         <v>27</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E55" t="s">
         <v>311</v>
       </c>
-      <c r="F55" s="11" t="s">
+      <c r="F55" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G55" s="11" t="s">
+      <c r="G55" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H55" s="5" t="s">
@@ -3727,15 +3734,15 @@
         <v>27</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E56" t="s">
         <v>316</v>
       </c>
-      <c r="F56" s="11" t="s">
+      <c r="F56" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G56" s="11" t="s">
+      <c r="G56" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H56" s="5" t="s">
@@ -3763,15 +3770,15 @@
         <v>27</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E57" t="s">
         <v>316</v>
       </c>
-      <c r="F57" s="11" t="s">
+      <c r="F57" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G57" s="11" t="s">
+      <c r="G57" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H57" s="5" t="s">
@@ -3799,15 +3806,15 @@
         <v>27</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E58" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E58" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="F58" s="11" t="s">
+      <c r="F58" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G58" s="11" t="s">
+      <c r="G58" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H58" s="5" t="s">
@@ -3835,15 +3842,15 @@
         <v>27</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E59" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E59" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="F59" s="11" t="s">
+      <c r="F59" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G59" s="11" t="s">
+      <c r="G59" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H59" s="5" t="s">
@@ -3871,15 +3878,15 @@
         <v>27</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E60" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="E60" s="8" t="s">
         <v>331</v>
       </c>
-      <c r="F60" s="11" t="s">
+      <c r="F60" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G60" s="11" t="s">
+      <c r="G60" s="9" t="s">
         <v>312</v>
       </c>
       <c r="H60" s="5" t="s">
@@ -3907,15 +3914,15 @@
         <v>60</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E61" t="s">
         <v>323</v>
       </c>
-      <c r="F61" s="11" t="s">
+      <c r="F61" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G61" s="11" t="s">
+      <c r="G61" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H61" s="5" t="s">
@@ -3943,15 +3950,15 @@
         <v>60</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E62" t="s">
         <v>323</v>
       </c>
-      <c r="F62" s="11" t="s">
+      <c r="F62" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G62" s="11" t="s">
+      <c r="G62" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H62" s="5" t="s">
@@ -3979,15 +3986,15 @@
         <v>60</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E63" t="s">
         <v>323</v>
       </c>
-      <c r="F63" s="11" t="s">
+      <c r="F63" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G63" s="11" t="s">
+      <c r="G63" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H63" s="5" t="s">
@@ -4015,15 +4022,15 @@
         <v>60</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E64" t="s">
         <v>326</v>
       </c>
-      <c r="F64" s="11" t="s">
+      <c r="F64" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G64" s="11" t="s">
+      <c r="G64" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H64" s="5" t="s">
@@ -4051,15 +4058,15 @@
         <v>60</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E65" t="s">
         <v>326</v>
       </c>
-      <c r="F65" s="11" t="s">
+      <c r="F65" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G65" s="11" t="s">
+      <c r="G65" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H65" s="5" t="s">
@@ -4087,15 +4094,15 @@
         <v>60</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E66" t="s">
         <v>330</v>
       </c>
-      <c r="F66" s="11" t="s">
+      <c r="F66" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G66" s="11" t="s">
+      <c r="G66" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H66" s="5" t="s">
@@ -4123,15 +4130,15 @@
         <v>60</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E67" t="s">
         <v>330</v>
       </c>
-      <c r="F67" s="11" t="s">
+      <c r="F67" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G67" s="11" t="s">
+      <c r="G67" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H67" s="5" t="s">
@@ -4159,15 +4166,15 @@
         <v>60</v>
       </c>
       <c r="D68" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E68" t="s">
         <v>330</v>
       </c>
-      <c r="F68" s="11" t="s">
+      <c r="F68" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G68" s="11" t="s">
+      <c r="G68" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H68" s="5" t="s">
@@ -4195,15 +4202,15 @@
         <v>60</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E69" t="s">
         <v>335</v>
       </c>
-      <c r="F69" s="11" t="s">
+      <c r="F69" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G69" s="11" t="s">
+      <c r="G69" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H69" s="5" t="s">
@@ -4231,15 +4238,15 @@
         <v>60</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E70" t="s">
         <v>335</v>
       </c>
-      <c r="F70" s="11" t="s">
+      <c r="F70" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G70" s="11" t="s">
+      <c r="G70" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H70" s="5" t="s">
@@ -4267,15 +4274,15 @@
         <v>60</v>
       </c>
       <c r="D71" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E71" t="s">
         <v>335</v>
       </c>
-      <c r="F71" s="11" t="s">
+      <c r="F71" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="G71" s="11" t="s">
+      <c r="G71" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H71" s="5" t="s">
@@ -4303,15 +4310,15 @@
         <v>14</v>
       </c>
       <c r="D72" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E72" t="s">
         <v>340</v>
       </c>
-      <c r="F72" s="11" t="s">
+      <c r="F72" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G72" s="11" t="s">
+      <c r="G72" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H72" s="5" t="s">
@@ -4339,15 +4346,15 @@
         <v>14</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E73" t="s">
         <v>340</v>
       </c>
-      <c r="F73" s="11" t="s">
+      <c r="F73" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G73" s="11" t="s">
+      <c r="G73" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H73" s="5" t="s">
@@ -4375,15 +4382,15 @@
         <v>14</v>
       </c>
       <c r="D74" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E74" t="s">
         <v>340</v>
       </c>
-      <c r="F74" s="11" t="s">
+      <c r="F74" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G74" s="11" t="s">
+      <c r="G74" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H74" s="5" t="s">
@@ -4411,15 +4418,15 @@
         <v>14</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E75" t="s">
         <v>340</v>
       </c>
-      <c r="F75" s="11" t="s">
+      <c r="F75" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G75" s="11" t="s">
+      <c r="G75" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H75" s="5" t="s">
@@ -4447,15 +4454,15 @@
         <v>14</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E76" t="s">
         <v>347</v>
       </c>
-      <c r="F76" s="11" t="s">
+      <c r="F76" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G76" s="11" t="s">
+      <c r="G76" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H76" s="5" t="s">
@@ -4483,15 +4490,15 @@
         <v>14</v>
       </c>
       <c r="D77" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E77" t="s">
         <v>347</v>
       </c>
-      <c r="F77" s="11" t="s">
+      <c r="F77" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G77" s="11" t="s">
+      <c r="G77" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H77" s="5" t="s">
@@ -4512,22 +4519,22 @@
       <c r="A78" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="B78" s="12" t="s">
+      <c r="B78" s="10" t="s">
         <v>346</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D78" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E78" t="s">
         <v>347</v>
       </c>
-      <c r="F78" s="11" t="s">
+      <c r="F78" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G78" s="11" t="s">
+      <c r="G78" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H78" s="5" t="s">
@@ -4555,15 +4562,15 @@
         <v>14</v>
       </c>
       <c r="D79" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E79" t="s">
         <v>347</v>
       </c>
-      <c r="F79" s="11" t="s">
+      <c r="F79" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G79" s="11" t="s">
+      <c r="G79" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H79" s="5" t="s">
@@ -4591,15 +4598,15 @@
         <v>14</v>
       </c>
       <c r="D80" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E80" t="s">
         <v>352</v>
       </c>
-      <c r="F80" s="11" t="s">
+      <c r="F80" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G80" s="11" t="s">
+      <c r="G80" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H80" s="5" t="s">
@@ -4627,15 +4634,15 @@
         <v>14</v>
       </c>
       <c r="D81" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E81" t="s">
         <v>352</v>
       </c>
-      <c r="F81" s="11" t="s">
+      <c r="F81" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G81" s="11" t="s">
+      <c r="G81" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H81" s="5" t="s">
@@ -4663,15 +4670,15 @@
         <v>14</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E82" t="s">
         <v>352</v>
       </c>
-      <c r="F82" s="11" t="s">
+      <c r="F82" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G82" s="11" t="s">
+      <c r="G82" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H82" s="5" t="s">
@@ -4699,15 +4706,15 @@
         <v>14</v>
       </c>
       <c r="D83" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E83" t="s">
         <v>352</v>
       </c>
-      <c r="F83" s="11" t="s">
+      <c r="F83" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G83" s="11" t="s">
+      <c r="G83" s="9" t="s">
         <v>341</v>
       </c>
       <c r="H83" s="5" t="s">
@@ -4728,22 +4735,22 @@
       <c r="A84" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="B84" s="12" t="s">
+      <c r="B84" s="10" t="s">
         <v>353</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D84" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E84" t="s">
         <v>356</v>
       </c>
-      <c r="F84" s="11" t="s">
+      <c r="F84" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G84" s="11" t="s">
+      <c r="G84" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H84" s="5" t="s">
@@ -4764,22 +4771,22 @@
       <c r="A85" s="4" t="s">
         <v>187</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="10" t="s">
         <v>354</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D85" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E85" t="s">
         <v>356</v>
       </c>
-      <c r="F85" s="11" t="s">
+      <c r="F85" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G85" s="11" t="s">
+      <c r="G85" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H85" s="5" t="s">
@@ -4800,22 +4807,22 @@
       <c r="A86" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="B86" s="12" t="s">
+      <c r="B86" s="10" t="s">
         <v>355</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>60</v>
       </c>
       <c r="D86" s="5" t="s">
-        <v>15</v>
+        <v>357</v>
       </c>
       <c r="E86" t="s">
         <v>356</v>
       </c>
-      <c r="F86" s="11" t="s">
+      <c r="F86" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="G86" s="11" t="s">
+      <c r="G86" s="9" t="s">
         <v>261</v>
       </c>
       <c r="H86" s="5" t="s">
@@ -4890,14 +4897,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
@@ -5021,7 +5028,7 @@
       <c r="B3" t="s">
         <v>210</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>242</v>
       </c>
       <c r="D3" t="s">
@@ -5038,7 +5045,7 @@
       <c r="B4" t="s">
         <v>213</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="8" t="s">
         <v>282</v>
       </c>
       <c r="D4" t="s">
@@ -5055,7 +5062,7 @@
       <c r="B5" t="s">
         <v>216</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="8" t="s">
         <v>313</v>
       </c>
       <c r="D5" t="s">
@@ -5077,7 +5084,7 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="8" t="s">
         <v>228</v>
       </c>
       <c r="D7" t="s">
@@ -5088,7 +5095,7 @@
       </c>
     </row>
     <row r="8" spans="1:5">
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="8" t="s">
         <v>342</v>
       </c>
       <c r="E8" t="s">

</xml_diff>

<commit_message>
Use Excel master for cards and filters
</commit_message>
<xml_diff>
--- a/card_master.xlsx
+++ b/card_master.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\平石　美帆\aikatsu-encore-manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{971C5BD4-EA63-432E-AA50-F41212D003B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F8F20B4-E0BA-44FA-A7F4-9C41BA5FDE0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="357">
   <si>
     <t>カード番号</t>
   </si>
@@ -1259,13 +1259,6 @@
   </si>
   <si>
     <t>イエローブロッサムコーデ</t>
-    <phoneticPr fontId="5"/>
-  </si>
-  <si>
-    <t>第一弾</t>
-    <rPh sb="0" eb="3">
-      <t>ダイイチダン</t>
-    </rPh>
     <phoneticPr fontId="5"/>
   </si>
 </sst>
@@ -1781,8 +1774,8 @@
       <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>357</v>
+      <c r="D2" s="5">
+        <v>1</v>
       </c>
       <c r="E2" t="s">
         <v>233</v>
@@ -1821,8 +1814,8 @@
       <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>357</v>
+      <c r="D3" s="5">
+        <v>1</v>
       </c>
       <c r="E3" t="s">
         <v>233</v>
@@ -1861,8 +1854,8 @@
       <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="5" t="s">
-        <v>357</v>
+      <c r="D4" s="5">
+        <v>1</v>
       </c>
       <c r="E4" t="s">
         <v>233</v>
@@ -1897,8 +1890,8 @@
       <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>357</v>
+      <c r="D5" s="5">
+        <v>1</v>
       </c>
       <c r="E5" t="s">
         <v>233</v>
@@ -1933,8 +1926,8 @@
       <c r="C6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>357</v>
+      <c r="D6" s="5">
+        <v>1</v>
       </c>
       <c r="E6" t="s">
         <v>238</v>
@@ -1969,8 +1962,8 @@
       <c r="C7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>357</v>
+      <c r="D7" s="5">
+        <v>1</v>
       </c>
       <c r="E7" t="s">
         <v>238</v>
@@ -2005,8 +1998,8 @@
       <c r="C8" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>357</v>
+      <c r="D8" s="5">
+        <v>1</v>
       </c>
       <c r="E8" t="s">
         <v>238</v>
@@ -2041,8 +2034,8 @@
       <c r="C9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>357</v>
+      <c r="D9" s="5">
+        <v>1</v>
       </c>
       <c r="E9" t="s">
         <v>238</v>
@@ -2077,8 +2070,8 @@
       <c r="C10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>357</v>
+      <c r="D10" s="5">
+        <v>1</v>
       </c>
       <c r="E10" t="s">
         <v>240</v>
@@ -2113,8 +2106,8 @@
       <c r="C11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>357</v>
+      <c r="D11" s="5">
+        <v>1</v>
       </c>
       <c r="E11" t="s">
         <v>246</v>
@@ -2149,8 +2142,8 @@
       <c r="C12" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>357</v>
+      <c r="D12" s="5">
+        <v>1</v>
       </c>
       <c r="E12" t="s">
         <v>246</v>
@@ -2185,8 +2178,8 @@
       <c r="C13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>357</v>
+      <c r="D13" s="5">
+        <v>1</v>
       </c>
       <c r="E13" t="s">
         <v>246</v>
@@ -2221,8 +2214,8 @@
       <c r="C14" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>357</v>
+      <c r="D14" s="5">
+        <v>1</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>251</v>
@@ -2257,8 +2250,8 @@
       <c r="C15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>357</v>
+      <c r="D15" s="5">
+        <v>1</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>251</v>
@@ -2293,8 +2286,8 @@
       <c r="C16" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>357</v>
+      <c r="D16" s="5">
+        <v>1</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>251</v>
@@ -2329,8 +2322,8 @@
       <c r="C17" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D17" s="5" t="s">
-        <v>357</v>
+      <c r="D17" s="5">
+        <v>1</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>251</v>
@@ -2365,8 +2358,8 @@
       <c r="C18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>357</v>
+      <c r="D18" s="5">
+        <v>1</v>
       </c>
       <c r="E18" t="s">
         <v>257</v>
@@ -2401,8 +2394,8 @@
       <c r="C19" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="5" t="s">
-        <v>357</v>
+      <c r="D19" s="5">
+        <v>1</v>
       </c>
       <c r="E19" t="s">
         <v>257</v>
@@ -2437,8 +2430,8 @@
       <c r="C20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>357</v>
+      <c r="D20" s="5">
+        <v>1</v>
       </c>
       <c r="E20" t="s">
         <v>257</v>
@@ -2473,8 +2466,8 @@
       <c r="C21" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>357</v>
+      <c r="D21" s="5">
+        <v>1</v>
       </c>
       <c r="E21" t="s">
         <v>257</v>
@@ -2509,8 +2502,8 @@
       <c r="C22" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>357</v>
+      <c r="D22" s="5">
+        <v>1</v>
       </c>
       <c r="E22" t="s">
         <v>260</v>
@@ -2545,8 +2538,8 @@
       <c r="C23" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>357</v>
+      <c r="D23" s="5">
+        <v>1</v>
       </c>
       <c r="E23" t="s">
         <v>260</v>
@@ -2581,8 +2574,8 @@
       <c r="C24" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>357</v>
+      <c r="D24" s="5">
+        <v>1</v>
       </c>
       <c r="E24" t="s">
         <v>260</v>
@@ -2617,8 +2610,8 @@
       <c r="C25" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>357</v>
+      <c r="D25" s="5">
+        <v>1</v>
       </c>
       <c r="E25" t="s">
         <v>265</v>
@@ -2653,8 +2646,8 @@
       <c r="C26" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="5" t="s">
-        <v>357</v>
+      <c r="D26" s="5">
+        <v>1</v>
       </c>
       <c r="E26" t="s">
         <v>265</v>
@@ -2689,8 +2682,8 @@
       <c r="C27" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>357</v>
+      <c r="D27" s="5">
+        <v>1</v>
       </c>
       <c r="E27" t="s">
         <v>265</v>
@@ -2725,8 +2718,8 @@
       <c r="C28" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="5" t="s">
-        <v>357</v>
+      <c r="D28" s="5">
+        <v>1</v>
       </c>
       <c r="E28" t="s">
         <v>270</v>
@@ -2761,8 +2754,8 @@
       <c r="C29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>357</v>
+      <c r="D29" s="5">
+        <v>1</v>
       </c>
       <c r="E29" t="s">
         <v>270</v>
@@ -2797,8 +2790,8 @@
       <c r="C30" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>357</v>
+      <c r="D30" s="5">
+        <v>1</v>
       </c>
       <c r="E30" t="s">
         <v>270</v>
@@ -2833,8 +2826,8 @@
       <c r="C31" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>357</v>
+      <c r="D31" s="5">
+        <v>1</v>
       </c>
       <c r="E31" t="s">
         <v>273</v>
@@ -2869,8 +2862,8 @@
       <c r="C32" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D32" s="5" t="s">
-        <v>357</v>
+      <c r="D32" s="5">
+        <v>1</v>
       </c>
       <c r="E32" t="s">
         <v>275</v>
@@ -2905,8 +2898,8 @@
       <c r="C33" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D33" s="5" t="s">
-        <v>357</v>
+      <c r="D33" s="5">
+        <v>1</v>
       </c>
       <c r="E33" t="s">
         <v>278</v>
@@ -2941,8 +2934,8 @@
       <c r="C34" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="5" t="s">
-        <v>357</v>
+      <c r="D34" s="5">
+        <v>1</v>
       </c>
       <c r="E34" t="s">
         <v>280</v>
@@ -2977,8 +2970,8 @@
       <c r="C35" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="5" t="s">
-        <v>357</v>
+      <c r="D35" s="5">
+        <v>1</v>
       </c>
       <c r="E35" t="s">
         <v>280</v>
@@ -3013,8 +3006,8 @@
       <c r="C36" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D36" s="5" t="s">
-        <v>357</v>
+      <c r="D36" s="5">
+        <v>1</v>
       </c>
       <c r="E36" t="s">
         <v>280</v>
@@ -3049,8 +3042,8 @@
       <c r="C37" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D37" s="5" t="s">
-        <v>357</v>
+      <c r="D37" s="5">
+        <v>1</v>
       </c>
       <c r="E37" t="s">
         <v>280</v>
@@ -3085,8 +3078,8 @@
       <c r="C38" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D38" s="5" t="s">
-        <v>357</v>
+      <c r="D38" s="5">
+        <v>1</v>
       </c>
       <c r="E38" t="s">
         <v>287</v>
@@ -3121,8 +3114,8 @@
       <c r="C39" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>357</v>
+      <c r="D39" s="5">
+        <v>1</v>
       </c>
       <c r="E39" t="s">
         <v>289</v>
@@ -3157,8 +3150,8 @@
       <c r="C40" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>357</v>
+      <c r="D40" s="5">
+        <v>1</v>
       </c>
       <c r="E40" t="s">
         <v>289</v>
@@ -3193,8 +3186,8 @@
       <c r="C41" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D41" s="5" t="s">
-        <v>357</v>
+      <c r="D41" s="5">
+        <v>1</v>
       </c>
       <c r="E41" t="s">
         <v>289</v>
@@ -3229,8 +3222,8 @@
       <c r="C42" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="5" t="s">
-        <v>357</v>
+      <c r="D42" s="5">
+        <v>1</v>
       </c>
       <c r="E42" t="s">
         <v>295</v>
@@ -3265,8 +3258,8 @@
       <c r="C43" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>357</v>
+      <c r="D43" s="5">
+        <v>1</v>
       </c>
       <c r="E43" t="s">
         <v>295</v>
@@ -3301,8 +3294,8 @@
       <c r="C44" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>357</v>
+      <c r="D44" s="5">
+        <v>1</v>
       </c>
       <c r="E44" t="s">
         <v>295</v>
@@ -3337,8 +3330,8 @@
       <c r="C45" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D45" s="5" t="s">
-        <v>357</v>
+      <c r="D45" s="5">
+        <v>1</v>
       </c>
       <c r="E45" t="s">
         <v>298</v>
@@ -3373,8 +3366,8 @@
       <c r="C46" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D46" s="5" t="s">
-        <v>357</v>
+      <c r="D46" s="5">
+        <v>1</v>
       </c>
       <c r="E46" t="s">
         <v>298</v>
@@ -3409,8 +3402,8 @@
       <c r="C47" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D47" s="5" t="s">
-        <v>357</v>
+      <c r="D47" s="5">
+        <v>1</v>
       </c>
       <c r="E47" t="s">
         <v>298</v>
@@ -3445,8 +3438,8 @@
       <c r="C48" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>357</v>
+      <c r="D48" s="5">
+        <v>1</v>
       </c>
       <c r="E48" t="s">
         <v>303</v>
@@ -3481,8 +3474,8 @@
       <c r="C49" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D49" s="5" t="s">
-        <v>357</v>
+      <c r="D49" s="5">
+        <v>1</v>
       </c>
       <c r="E49" t="s">
         <v>303</v>
@@ -3517,8 +3510,8 @@
       <c r="C50" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D50" s="5" t="s">
-        <v>357</v>
+      <c r="D50" s="5">
+        <v>1</v>
       </c>
       <c r="E50" t="s">
         <v>303</v>
@@ -3553,8 +3546,8 @@
       <c r="C51" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>357</v>
+      <c r="D51" s="5">
+        <v>1</v>
       </c>
       <c r="E51" t="s">
         <v>305</v>
@@ -3589,8 +3582,8 @@
       <c r="C52" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D52" s="5" t="s">
-        <v>357</v>
+      <c r="D52" s="5">
+        <v>1</v>
       </c>
       <c r="E52" t="s">
         <v>307</v>
@@ -3625,8 +3618,8 @@
       <c r="C53" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>357</v>
+      <c r="D53" s="5">
+        <v>1</v>
       </c>
       <c r="E53" t="s">
         <v>307</v>
@@ -3661,8 +3654,8 @@
       <c r="C54" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D54" s="5" t="s">
-        <v>357</v>
+      <c r="D54" s="5">
+        <v>1</v>
       </c>
       <c r="E54" t="s">
         <v>311</v>
@@ -3697,8 +3690,8 @@
       <c r="C55" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>357</v>
+      <c r="D55" s="5">
+        <v>1</v>
       </c>
       <c r="E55" t="s">
         <v>311</v>
@@ -3733,8 +3726,8 @@
       <c r="C56" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D56" s="5" t="s">
-        <v>357</v>
+      <c r="D56" s="5">
+        <v>1</v>
       </c>
       <c r="E56" t="s">
         <v>316</v>
@@ -3769,8 +3762,8 @@
       <c r="C57" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D57" s="5" t="s">
-        <v>357</v>
+      <c r="D57" s="5">
+        <v>1</v>
       </c>
       <c r="E57" t="s">
         <v>316</v>
@@ -3805,8 +3798,8 @@
       <c r="C58" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D58" s="5" t="s">
-        <v>357</v>
+      <c r="D58" s="5">
+        <v>1</v>
       </c>
       <c r="E58" s="8" t="s">
         <v>331</v>
@@ -3841,8 +3834,8 @@
       <c r="C59" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D59" s="5" t="s">
-        <v>357</v>
+      <c r="D59" s="5">
+        <v>1</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>331</v>
@@ -3877,8 +3870,8 @@
       <c r="C60" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D60" s="5" t="s">
-        <v>357</v>
+      <c r="D60" s="5">
+        <v>1</v>
       </c>
       <c r="E60" s="8" t="s">
         <v>331</v>
@@ -3913,8 +3906,8 @@
       <c r="C61" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D61" s="5" t="s">
-        <v>357</v>
+      <c r="D61" s="5">
+        <v>1</v>
       </c>
       <c r="E61" t="s">
         <v>323</v>
@@ -3949,8 +3942,8 @@
       <c r="C62" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D62" s="5" t="s">
-        <v>357</v>
+      <c r="D62" s="5">
+        <v>1</v>
       </c>
       <c r="E62" t="s">
         <v>323</v>
@@ -3985,8 +3978,8 @@
       <c r="C63" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D63" s="5" t="s">
-        <v>357</v>
+      <c r="D63" s="5">
+        <v>1</v>
       </c>
       <c r="E63" t="s">
         <v>323</v>
@@ -4021,8 +4014,8 @@
       <c r="C64" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D64" s="5" t="s">
-        <v>357</v>
+      <c r="D64" s="5">
+        <v>1</v>
       </c>
       <c r="E64" t="s">
         <v>326</v>
@@ -4057,8 +4050,8 @@
       <c r="C65" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>357</v>
+      <c r="D65" s="5">
+        <v>1</v>
       </c>
       <c r="E65" t="s">
         <v>326</v>
@@ -4093,8 +4086,8 @@
       <c r="C66" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D66" s="5" t="s">
-        <v>357</v>
+      <c r="D66" s="5">
+        <v>1</v>
       </c>
       <c r="E66" t="s">
         <v>330</v>
@@ -4129,8 +4122,8 @@
       <c r="C67" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D67" s="5" t="s">
-        <v>357</v>
+      <c r="D67" s="5">
+        <v>1</v>
       </c>
       <c r="E67" t="s">
         <v>330</v>
@@ -4165,8 +4158,8 @@
       <c r="C68" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D68" s="5" t="s">
-        <v>357</v>
+      <c r="D68" s="5">
+        <v>1</v>
       </c>
       <c r="E68" t="s">
         <v>330</v>
@@ -4201,8 +4194,8 @@
       <c r="C69" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D69" s="5" t="s">
-        <v>357</v>
+      <c r="D69" s="5">
+        <v>1</v>
       </c>
       <c r="E69" t="s">
         <v>335</v>
@@ -4237,8 +4230,8 @@
       <c r="C70" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D70" s="5" t="s">
-        <v>357</v>
+      <c r="D70" s="5">
+        <v>1</v>
       </c>
       <c r="E70" t="s">
         <v>335</v>
@@ -4273,8 +4266,8 @@
       <c r="C71" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D71" s="5" t="s">
-        <v>357</v>
+      <c r="D71" s="5">
+        <v>1</v>
       </c>
       <c r="E71" t="s">
         <v>335</v>
@@ -4309,8 +4302,8 @@
       <c r="C72" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D72" s="5" t="s">
-        <v>357</v>
+      <c r="D72" s="5">
+        <v>1</v>
       </c>
       <c r="E72" t="s">
         <v>340</v>
@@ -4345,8 +4338,8 @@
       <c r="C73" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D73" s="5" t="s">
-        <v>357</v>
+      <c r="D73" s="5">
+        <v>1</v>
       </c>
       <c r="E73" t="s">
         <v>340</v>
@@ -4381,8 +4374,8 @@
       <c r="C74" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D74" s="5" t="s">
-        <v>357</v>
+      <c r="D74" s="5">
+        <v>1</v>
       </c>
       <c r="E74" t="s">
         <v>340</v>
@@ -4417,8 +4410,8 @@
       <c r="C75" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D75" s="5" t="s">
-        <v>357</v>
+      <c r="D75" s="5">
+        <v>1</v>
       </c>
       <c r="E75" t="s">
         <v>340</v>
@@ -4453,8 +4446,8 @@
       <c r="C76" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D76" s="5" t="s">
-        <v>357</v>
+      <c r="D76" s="5">
+        <v>1</v>
       </c>
       <c r="E76" t="s">
         <v>347</v>
@@ -4489,8 +4482,8 @@
       <c r="C77" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D77" s="5" t="s">
-        <v>357</v>
+      <c r="D77" s="5">
+        <v>1</v>
       </c>
       <c r="E77" t="s">
         <v>347</v>
@@ -4525,8 +4518,8 @@
       <c r="C78" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D78" s="5" t="s">
-        <v>357</v>
+      <c r="D78" s="5">
+        <v>1</v>
       </c>
       <c r="E78" t="s">
         <v>347</v>
@@ -4561,8 +4554,8 @@
       <c r="C79" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D79" s="5" t="s">
-        <v>357</v>
+      <c r="D79" s="5">
+        <v>1</v>
       </c>
       <c r="E79" t="s">
         <v>347</v>
@@ -4597,8 +4590,8 @@
       <c r="C80" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D80" s="5" t="s">
-        <v>357</v>
+      <c r="D80" s="5">
+        <v>1</v>
       </c>
       <c r="E80" t="s">
         <v>352</v>
@@ -4633,8 +4626,8 @@
       <c r="C81" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D81" s="5" t="s">
-        <v>357</v>
+      <c r="D81" s="5">
+        <v>1</v>
       </c>
       <c r="E81" t="s">
         <v>352</v>
@@ -4669,8 +4662,8 @@
       <c r="C82" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D82" s="5" t="s">
-        <v>357</v>
+      <c r="D82" s="5">
+        <v>1</v>
       </c>
       <c r="E82" t="s">
         <v>352</v>
@@ -4705,8 +4698,8 @@
       <c r="C83" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D83" s="5" t="s">
-        <v>357</v>
+      <c r="D83" s="5">
+        <v>1</v>
       </c>
       <c r="E83" t="s">
         <v>352</v>
@@ -4741,8 +4734,8 @@
       <c r="C84" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D84" s="5" t="s">
-        <v>357</v>
+      <c r="D84" s="5">
+        <v>1</v>
       </c>
       <c r="E84" t="s">
         <v>356</v>
@@ -4777,8 +4770,8 @@
       <c r="C85" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D85" s="5" t="s">
-        <v>357</v>
+      <c r="D85" s="5">
+        <v>1</v>
       </c>
       <c r="E85" t="s">
         <v>356</v>
@@ -4813,8 +4806,8 @@
       <c r="C86" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D86" s="5" t="s">
-        <v>357</v>
+      <c r="D86" s="5">
+        <v>1</v>
       </c>
       <c r="E86" t="s">
         <v>356</v>

</xml_diff>